<commit_message>
feat: Connect contact enquiries directly to dynamic Excel database export and add verification test
</commit_message>
<xml_diff>
--- a/exports/CSK_Contact_Enquiries_Database.xlsx
+++ b/exports/CSK_Contact_Enquiries_Database.xlsx
@@ -100,126 +100,336 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-10T11:45:00Z</t>
+          <t>2026-10-13T12:09:50.140150+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10/10/2026, 6:45:00 AM</t>
+          <t>10/13/2026, 05:39:50 PM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Marcus Campbell</t>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>marcus@example.ky</t>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Corporate Sponsorship &amp; Brand Partnership</t>
+          <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Looking to discuss CSK corporate jersey sponsorship for the 2026/27 Super League season.</t>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Verified Website Submission</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Rahul Garg (Club Captain)</t>
+          <t>Committee Review</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-10T10:30:00Z</t>
+          <t>2026-10-13T12:08:22.626Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10/10/2026, 5:30:00 AM</t>
+          <t>10/13/2026, 05:38:22 PM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dave Robinson</t>
+          <t>Sahil Singh</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dave.r@example.ky</t>
+          <t>sahil.singh.trial@caymansuperkings.ky</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Youth Academy Registration (Ages 10–18)</t>
+          <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Interested in enrolling two youth players (under-15) for weekly coaching sessions.</t>
+          <t>Enquiring regarding upcoming open bowling trials for senior squad selection at Smith Road Oval.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Verified Website Submission</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Majin Paul (Team Manager)</t>
+          <t>Rahul Garg (Captain)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-10-10T11:45:00Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10/10/2026, 6:45:00 AM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Marcus Campbell</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>marcus@example.ky</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Corporate Sponsorship &amp; Brand Partnership</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Looking to discuss CSK corporate jersey sponsorship for the 2026/27 Super League season.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>In Review</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rahul Garg (Club Captain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:30:00Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10/10/2026, 5:30:00 AM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dave Robinson</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>dave.r@example.ky</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Youth Academy Registration (Ages 10–18)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Interested in enrolling two youth players (under-15) for weekly coaching sessions.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Majin Paul (Team Manager)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>2026-10-09T18:15:00Z</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>09/10/2026, 1:15:00 PM</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Sarah Jenkins</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>sarah.j@caymanports.ky</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>General Club Enquiry</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Inquiry regarding upcoming tournament schedule at Smith Road Oval and match ticketing.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Christopher Balraj (Co-Founder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:08:46.492Z</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/13/2026, 5:38:46 PM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Node API Test User</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>node.test@caymansuperkings.ky</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Corporate Sponsorship</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Testing Node.js contact-store integration with Excel generator</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Verified API Test</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Committee Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:08:22.626705+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/13/2026, 05:38:22 PM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Senior Squad Trials &amp; Recruitment</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Verified Website Submission</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Committee Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:07:08.088648Z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/13/2026, 05:37:08 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Senior Squad Trials &amp; Recruitment</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Verified Website Submission</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Committee Review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify and test Contact Page & Youth Academy form Excel database storage pipeline and add download endpoints
</commit_message>
<xml_diff>
--- a/exports/CSK_Contact_Enquiries_Database.xlsx
+++ b/exports/CSK_Contact_Enquiries_Database.xlsx
@@ -100,334 +100,466 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-13T12:09:50.140150+00:00</t>
+          <t>2026-10-14T15:48:58.444318+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10/13/2026, 05:39:50 PM</t>
+          <t>10/14/2026, 09:18:58 PM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sahil Singh (Player Trial Enquiry)</t>
+          <t>Michael Campbell (Contact Page Submission)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>sahil.singh.test@caymansuperkings.ky</t>
+          <t>michael.campbell@candw.ky</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Squad Trials &amp; Recruitment</t>
+          <t>Senior Squad Trials &amp; Corporate Partnership</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
+          <t>Enquiry submitted via contact.html regarding 2026/27 premier league trials and sponsor packages.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Verified Website Submission</t>
+          <t>Verified Contact Page Submission</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Committee Review</t>
+          <t>Rahul Garg (Club Captain)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-13T12:08:22.626Z</t>
+          <t>2026-10-14T15:48:58.444318+00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10/13/2026, 05:38:22 PM</t>
+          <t>10/14/2026, 09:18:58 PM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sahil Singh</t>
+          <t>David Miller (Youth Parent)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>sahil.singh.trial@caymansuperkings.ky</t>
+          <t>david.miller@caymanparent.ky</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Squad Trials &amp; Recruitment</t>
+          <t>Youth Academy Enrollment - Leo Miller, Age 11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Enquiring regarding upcoming open bowling trials for senior squad selection at Smith Road Oval.</t>
+          <t>[YOUTH ACADEMY ENROLLMENT]
+• Parent/Guardian: David Miller
+• Child Info &amp; Age: Leo Miller, Age 11
+• Phone / WhatsApp: +1 (345) 925-8844
+• Email: david.miller@caymanparent.ky
+• Experience Level: Intermediate
+• Training Ground: Smith Road Oval, George Town</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Verified Website Submission</t>
+          <t>Verified Youth Academy Enrollment</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rahul Garg (Captain)</t>
+          <t>Academy Coordinator</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-10T11:45:00Z</t>
+          <t>2026-10-14T15:48:04.714106+00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/10/2026, 6:45:00 AM</t>
+          <t>10/14/2026, 09:18:04 PM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Marcus Campbell</t>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>marcus@example.ky</t>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Corporate Sponsorship &amp; Brand Partnership</t>
+          <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Looking to discuss CSK corporate jersey sponsorship for the 2026/27 Super League season.</t>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Verified Website Submission</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Rahul Garg (Club Captain)</t>
+          <t>Committee Review</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-10T10:30:00Z</t>
+          <t>2026-10-13T12:09:50.140150+00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10/10/2026, 5:30:00 AM</t>
+          <t>10/13/2026, 05:39:50 PM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dave Robinson</t>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>dave.r@example.ky</t>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Youth Academy Registration (Ages 10–18)</t>
+          <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Interested in enrolling two youth players (under-15) for weekly coaching sessions.</t>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Verified Website Submission</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Majin Paul (Team Manager)</t>
+          <t>Committee Review</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-09T18:15:00Z</t>
+          <t>2026-10-13T12:08:22.626Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>09/10/2026, 1:15:00 PM</t>
+          <t>10/13/2026, 05:38:22 PM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sarah Jenkins</t>
+          <t>Sahil Singh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sarah.j@caymanports.ky</t>
+          <t>sahil.singh.trial@caymansuperkings.ky</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>General Club Enquiry</t>
+          <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Inquiry regarding upcoming tournament schedule at Smith Road Oval and match ticketing.</t>
+          <t>Enquiring regarding upcoming open bowling trials for senior squad selection at Smith Road Oval.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Contacted</t>
+          <t>Verified Website Submission</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Christopher Balraj (Co-Founder)</t>
+          <t>Rahul Garg (Captain)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-13T12:08:46.492Z</t>
+          <t>2026-10-10T11:45:00Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10/13/2026, 5:38:46 PM</t>
+          <t>10/10/2026, 6:45:00 AM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Node API Test User</t>
+          <t>Marcus Campbell</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>node.test@caymansuperkings.ky</t>
+          <t>marcus@example.ky</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Corporate Sponsorship</t>
+          <t>Corporate Sponsorship &amp; Brand Partnership</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Testing Node.js contact-store integration with Excel generator</t>
+          <t>Looking to discuss CSK corporate jersey sponsorship for the 2026/27 Super League season.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Verified API Test</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Committee Review</t>
+          <t>Rahul Garg (Club Captain)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-13T12:08:22.626705+00:00</t>
+          <t>2026-10-10T10:30:00Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/13/2026, 05:38:22 PM</t>
+          <t>10/10/2026, 5:30:00 AM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sahil Singh (Player Trial Enquiry)</t>
+          <t>Dave Robinson</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>sahil.singh.test@caymansuperkings.ky</t>
+          <t>dave.r@example.ky</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Squad Trials &amp; Recruitment</t>
+          <t>Youth Academy Registration (Ages 10–18)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
+          <t>Interested in enrolling two youth players (under-15) for weekly coaching sessions.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Verified Website Submission</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Committee Review</t>
+          <t>Majin Paul (Team Manager)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>2026-10-09T18:15:00Z</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09/10/2026, 1:15:00 PM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sarah.j@caymanports.ky</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>General Club Enquiry</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Inquiry regarding upcoming tournament schedule at Smith Road Oval and match ticketing.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Contacted</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Christopher Balraj (Co-Founder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:08:46.492Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/13/2026, 5:38:46 PM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Node API Test User</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>node.test@caymansuperkings.ky</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Corporate Sponsorship</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Testing Node.js contact-store integration with Excel generator</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Verified API Test</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Committee Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:08:22.626705+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10/13/2026, 05:38:22 PM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sahil Singh (Player Trial Enquiry)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>sahil.singh.test@caymansuperkings.ky</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Senior Squad Trials &amp; Recruitment</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Verified Website Submission</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Committee Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2026-10-13T12:07:08.088648Z</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>10/13/2026, 05:37:08 PM</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Sahil Singh (Player Trial Enquiry)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>sahil.singh.test@caymansuperkings.ky</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Senior Squad Trials &amp; Recruitment</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Verified Website Submission</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Committee Review</t>
         </is>

</xml_diff>

<commit_message>
Add David Warner Cayman photo to gallery and hide partnership tiers section on partner page
</commit_message>
<xml_diff>
--- a/exports/CSK_Contact_Enquiries_Database.xlsx
+++ b/exports/CSK_Contact_Enquiries_Database.xlsx
@@ -439,132 +439,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-10-13T12:08:46.492Z</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>10/13/2026, 5:38:46 PM</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Node API Test User</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>node.test@caymansuperkings.ky</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Corporate Sponsorship</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Testing Node.js contact-store integration with Excel generator</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Verified API Test</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Committee Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-10-13T12:08:22.626705+00:00</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10/13/2026, 05:38:22 PM</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Sahil Singh (Player Trial Enquiry)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>sahil.singh.test@caymansuperkings.ky</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Senior Squad Trials &amp; Recruitment</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Verified Website Submission</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Committee Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-10-13T12:07:08.088648Z</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>10/13/2026, 05:37:08 PM</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Sahil Singh (Player Trial Enquiry)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>sahil.singh.test@caymansuperkings.ky</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Senior Squad Trials &amp; Recruitment</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Testing automated verification that contact page enquiries are accurately saved in Excel (.xlsx) database.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Verified Website Submission</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Committee Review</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>